<commit_message>
refactor(motivos): Passo 3 — planilha e código alinhados à matriz aprovada
6 textos renomeados no código para bater com os nomes aprovados na planilha:
- "Finaud escreveu ao cliente" → "Finaud fez pergunta — aguarda resposta"
- "Finaud acusou recibo" → "Cliente enviou informações e extratos"
- "Finaud recebeu arquivos do cliente" → "Cliente enviou informações e extratos"
- "Finaud escreveu — aguarda retorno do cliente" → "Finaud fez pergunta — aguarda resposta"
- "Cliente informou aceite do BACEN" → "Confirmação de entrega no BACEN"
- "Cliente escreveu — aguarda resposta da Finaud" → "Cliente fez pergunta — aguarda resposta da Finaud"

Planilha: linha nova (BANVOX), termos atualizados em 4 linhas.
Testes atualizados para refletir os nomes corretos. 525 passed.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentações/matriz_classificacao_motivos.xlsx
+++ b/documentações/matriz_classificacao_motivos.xlsx
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -656,7 +656,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>"segue"; "seguem"; "conforme anexo"; "em anexo"; "encaminho"; "encaminhamos"; "estou enviando"</t>
+          <t>"segue"; "seguem"; "conforme anexo"; "em anexo"; "encaminho"; "encaminhamos"; "estou enviando"; "fyi"; "apenas confirmando"; "acabei de envi"; "pode seguir"; "houve compromissada"; "sem movimenta"; "anexo posições"; "anexo extratos"; "anexo arquivo"</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>"precisamos"; "necessitamos"; "gostaríamos"; "precisaria"; "peço que"; "favor"</t>
+          <t>"precisamos"; "necessitamos"; "gostaríamos"; "precisaria"; "peço que"; "favor"; "gentileza"; "poderia"; "preciso"; "pode enviar"; "por favor"; "seria possível"; "pode confirmar"; "pode verificar"; "algum retorno"; "conseguiu verificar"; "foi possível"; "me atualizar"; "reforçar"; "em atraso"; "consegue me confirmar"</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>"retornaremos em breve"; "retornaremos"; "retornarei"; "estamos verificando"; "estamos analisando"; "vamos verificar"; "em análise"; "em verificação"; "aguarde o retorno"; "assim que tiver"; "pedi para"; "pedimos para"; "estarei colocando"</t>
+          <t>"retornaremos em breve"; "retornaremos"; "retornarei"; "estamos verificando"; "estamos analisando"; "estamos investigando"; "verificaremos"; "analisaremos"; "vamos verificar"; "vamos analisar"; "nossa equipe técnica"; "equipe técnica irá"; "em análise"; "em verificação"; "aguarde o retorno"; "assim que tiver"; "pedi para"; "pedimos para"; "estarei colocando"</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -898,50 +898,50 @@
       </c>
     </row>
     <row r="9" ht="6" customHeight="1">
-      <c r="A9" s="9" t="inlineStr"/>
-      <c r="B9" s="9" t="inlineStr"/>
-      <c r="C9" s="9" t="inlineStr"/>
-      <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
-      <c r="G9" s="9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Aguardando Finaud</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BANVOX encaminhou alerta do BACEN sobre documento — aguarda análise da Finaud</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sistema recebeu alerta do BACEN encaminhado pela BANVOX — a Finaud precisa analisar o documento antes de agir</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Não — código</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="56" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>Aguardando Cliente</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Finaud solicitou extrato ou planilha — aguarda envio</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Finaud pediu um documento (extrato, planilha ou arquivo) ao cliente e aguarda o envio</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>"solicitamos encaminhar"; "solicitamos que encaminhe"; "solicitamos que envie"; "poderia encaminhar por gentileza"; "vou precisar"</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>27/08/2026</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>Ativa</t>
-        </is>
-      </c>
+      <c r="A10" s="9" t="inlineStr"/>
+      <c r="B10" s="9" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="9" t="inlineStr"/>
     </row>
     <row r="11" ht="56" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -951,17 +951,17 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Finaud deu orientação técnica — aguarda execução</t>
+          <t>Finaud solicitou extrato ou planilha — aguarda envio</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Finaud instruiu o cliente a realizar algum procedimento e aguarda que o cliente execute</t>
+          <t>Finaud pediu um documento (extrato, planilha ou arquivo) ao cliente e aguarda o envio</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>"orientamos que"; "verifique"</t>
+          <t>"solicitamos encaminhar"; "solicitamos que encaminhe"; "solicitamos que envie"; "poderia encaminhar por gentileza"; "vou precisar"</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -988,17 +988,17 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Finaud propôs reunião ou ligação — aguarda confirmação</t>
+          <t>Finaud deu orientação técnica — aguarda execução</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Finaud sugeriu um horário ou formato de reunião e aguarda o cliente confirmar</t>
+          <t>Finaud instruiu o cliente a realizar algum procedimento e aguarda que o cliente execute</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>"reunião"; "ligação"; "videoconferência"; "Teams"; "Meet"</t>
+          <t>"orientamos que"; "verifique"</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -1025,17 +1025,17 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Finaud fez pergunta — aguarda resposta</t>
+          <t>Finaud propôs reunião ou ligação — aguarda confirmação</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Finaud fez uma pergunta ao cliente e aguarda a resposta</t>
+          <t>Finaud sugeriu um horário ou formato de reunião e aguarda o cliente confirmar</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>"reunião"; "ligação"; "videoconferência"; "Teams"; "Meet"</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1043,9 +1043,9 @@
           <t>27/08/2026</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Não — código</t>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1062,27 +1062,27 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Cliente prometeu retornar com informações — aguarda retorno</t>
+          <t>Finaud fez pergunta — aguarda resposta</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Cliente avisou que vai enviar algo ou dar uma resposta — a bola está com o cliente</t>
+          <t>Finaud fez uma pergunta ao cliente e aguarda a resposta</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>"retornaremos"; "retornamos"; "retornarei"; "vamos analisar"; "e retorno"</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>29/08/2026</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Não — código</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1099,80 +1099,80 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
+          <t>Cliente prometeu retornar com informações — aguarda retorno</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Cliente avisou que vai enviar algo ou dar uma resposta — a bola está com o cliente</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>"retornaremos"; "retornamos"; "retornarei"; "vamos analisar"; "e retorno"; "entrarei em contato"</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="6" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Aguardando Cliente</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
           <t>Finaud enviou arquivo — aguarda retorno do cliente</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Finaud enviou um arquivo sem usar as frases-padrão de entrega — sistema não confirmou se é entrega final; aguarda manifestação do cliente</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>29/08/2026</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Não — código</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>Ativa</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="6" customHeight="1">
-      <c r="A16" s="9" t="inlineStr"/>
-      <c r="B16" s="9" t="inlineStr"/>
-      <c r="C16" s="9" t="inlineStr"/>
-      <c r="D16" s="9" t="inlineStr"/>
-      <c r="E16" s="9" t="inlineStr"/>
-      <c r="F16" s="9" t="inlineStr"/>
-      <c r="G16" s="9" t="inlineStr"/>
-    </row>
     <row r="17" ht="56" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Concluída</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Finaud concluiu a solicitação</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Finaud respondeu e encerrou a conversa sem pedir nada ao cliente — assunto resolvido</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>"segue em anexo"; "segue o arquivo"; "encaminhamos"; "conforme solicitado"; "procedemos com"; "enviamos"; "foi enviado"; "já está disponível"; "ok, enviado"</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>27/08/2026</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>Ativa</t>
-        </is>
-      </c>
+      <c r="A17" s="9" t="inlineStr"/>
+      <c r="B17" s="9" t="inlineStr"/>
+      <c r="C17" s="9" t="inlineStr"/>
+      <c r="D17" s="9" t="inlineStr"/>
+      <c r="E17" s="9" t="inlineStr"/>
+      <c r="F17" s="9" t="inlineStr"/>
+      <c r="G17" s="9" t="inlineStr"/>
     </row>
     <row r="18" ht="56" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -1182,17 +1182,17 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>Cliente agradeceu — problema resolvido</t>
+          <t>Finaud concluiu a solicitação</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Cliente respondeu com agradecimento ou confirmação e não fez nova pergunta nem enviou documento — assunto encerrado</t>
+          <t>Finaud respondeu e encerrou a conversa sem pedir nada ao cliente — assunto resolvido</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>"obrigado"; "obrigada"; "ok"; "de acordo"; "concordo"; "recebido"; "perfeito"; "valeu"; "confirmado"; "entendido"; "sem problemas"; "deu certo"; "funcionou"; "resolveu"</t>
+          <t>"segue em anexo"; "segue o arquivo"; "encaminhamos"; "conforme solicitado"; "procedemos com"; "enviamos"; "foi enviado"; "já está disponível"; "ok, enviado"</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1219,17 +1219,17 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Finaud entregou arquivo ao cliente</t>
+          <t>Cliente agradeceu — problema resolvido</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Finaud enviou um arquivo ao cliente com frases de entrega — entrega confirmada</t>
+          <t>Cliente respondeu com agradecimento ou confirmação e não fez nova pergunta nem enviou documento — assunto encerrado</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>"segue em anexo"; "segue o arquivo"; "encaminhamos"; "conforme solicitado"; "enviamos"</t>
+          <t>"obrigado"; "obrigada"; "ok"; "de acordo"; "concordo"; "recebido"; "perfeito"; "valeu"; "confirmado"; "entendido"; "sem problemas"; "deu certo"; "funcionou"; "resolveu"</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1256,83 +1256,121 @@
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
+          <t>Finaud entregou arquivo ao cliente</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Finaud enviou um arquivo ao cliente com frases de entrega — entrega confirmada</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>"segue em anexo"; "segue o arquivo"; "encaminhamos"; "conforme solicitado"; "enviamos"</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="6" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Concluída</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
           <t>Confirmação de entrega no BACEN</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Sistema detectou que arquivo foi transmitido ao BACEN — processo encerrado</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>"transmitido no BACEN"; "transmitida no BACEN"; "arquivo transmitido"</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>27/08/2026</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>Ativa</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="6" customHeight="1">
-      <c r="A21" s="9" t="inlineStr"/>
-      <c r="B21" s="9" t="inlineStr"/>
-      <c r="C21" s="9" t="inlineStr"/>
-      <c r="D21" s="9" t="inlineStr"/>
-      <c r="E21" s="9" t="inlineStr"/>
-      <c r="F21" s="9" t="inlineStr"/>
-      <c r="G21" s="9" t="inlineStr"/>
-    </row>
     <row r="22" ht="56" customHeight="1">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr"/>
+      <c r="B22" s="9" t="inlineStr"/>
+      <c r="C22" s="9" t="inlineStr"/>
+      <c r="D22" s="9" t="inlineStr"/>
+      <c r="E22" s="9" t="inlineStr"/>
+      <c r="F22" s="9" t="inlineStr"/>
+      <c r="G22" s="9" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>Sem Retorno</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>Sem retorno há [N] dias — aguarda retorno</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Prazo configurado passou sem nova mensagem do cliente ou da Finaud — thread marcada como inativa</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>29/08/2026</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Não — código</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>Ativa</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="48" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
+    <row r="24" ht="48" customHeight="1"/>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Legenda (tela do sistema): "Esta thread está [Status] com o motivo '[Motivo]' porque [Razão do motivo] — o sistema identificou os termos '[Termos]', regra desde [Criado em]."
 "Você gerencia? Sim" → você edita os termos, o motivo e a razão pela tela de manutenção.
@@ -1354,7 +1392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1877,6 +1915,141 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Cliente enviou informações e extratos — aguarda processamento</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Termos configuráveis</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>"segue"; "seguem"; "conforme anexo"; "em anexo"; "encaminho"; "encaminhamos"; "estou enviando"</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>"segue"; "seguem"; "conforme anexo"; "em anexo"; "encaminho"; "encaminhamos"; "estou enviando"; "fyi"; "apenas confirmando"; "acabei de envi"; "pode seguir"; "houve compromissada"; "sem movimenta"; "anexo posições"; "anexo extratos"; "anexo arquivo"</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cliente fez solicitação — aguarda ação da Finaud</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Termos configuráveis</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>"precisamos"; "necessitamos"; "gostaríamos"; "precisaria"; "peço que"; "favor"</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>"precisamos"; "necessitamos"; "gostaríamos"; "precisaria"; "peço que"; "favor"; "gentileza"; "poderia"; "preciso"; "pode enviar"; "por favor"; "seria possível"; "pode confirmar"; "pode verificar"; "algum retorno"; "conseguiu verificar"; "foi possível"; "me atualizar"; "reforçar"; "em atraso"; "consegue me confirmar"</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Finaud prometeu retornar</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Termos configuráveis</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>"retornaremos em breve"; "retornaremos"; "retornarei"; "estamos verificando"; "estamos analisando"; "vamos verificar"; "em análise"; "em verificação"; "aguarde o retorno"; "assim que tiver"; "pedi para"; "pedimos para"; "estarei colocando"</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>"retornaremos em breve"; "retornaremos"; "retornarei"; "estamos verificando"; "estamos analisando"; "estamos investigando"; "verificaremos"; "analisaremos"; "vamos verificar"; "vamos analisar"; "nossa equipe técnica"; "equipe técnica irá"; "em análise"; "em verificação"; "aguarde o retorno"; "assim que tiver"; "pedi para"; "pedimos para"; "estarei colocando"</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cliente prometeu retornar com informações — aguarda retorno</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Termos configuráveis</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>"retornaremos"; "retornamos"; "retornarei"; "vamos analisar"; "e retorno"</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>"retornaremos"; "retornamos"; "retornarei"; "vamos analisar"; "e retorno"; "entrarei em contato"</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BANVOX encaminhou alerta do BACEN sobre documento — aguarda análise da Finaud</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Criação</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Regra criada</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>